<commit_message>
Update HR agent 07 training logistics
</commit_message>
<xml_diff>
--- a/hragent/downloads/hragent-synthetic-data.xlsx
+++ b/hragent/downloads/hragent-synthetic-data.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04-interview-evaluation-assista" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05-campus-recruitment-assistant" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06-talent-persona-assistant" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-training-outline-assistant" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07-training-logistics-assistant" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08-ppt-script-assistant" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09-training-material-search-ass" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-question-bank-assistant" sheetId="11" state="visible" r:id="rId11"/>
@@ -717,7 +717,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>课程大纲生成助手</t>
+          <t>培训后勤工作助手</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -727,12 +727,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>培训设计</t>
+          <t>培训后勤</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>training-outline-assistant</t>
+          <t>training-logistics-assistant</t>
         </is>
       </c>
       <c r="F8" s="2" t="b">
@@ -10550,52 +10550,64 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>course_id</t>
+          <t>logistics_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>audience</t>
+          <t>training_event</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>course_topic</t>
+          <t>participant_group</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>learning_goal</t>
+          <t>participant_count</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>duration</t>
+          <t>delivery_mode</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>delivery_mode</t>
+          <t>material_status</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>assessment_requirement</t>
+          <t>venue_mode</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>equipment_need</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>risk_note</t>
         </is>
       </c>
     </row>
@@ -10607,32 +10619,40 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>新员工训练营后勤</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>新员工</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>HR数据分析入门</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>能够独立完成HR数据分析入门的基础操作，并说明关键风险边界。</t>
-        </is>
+      <c r="D2" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>90分钟</t>
+          <t>线上直播</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>线上直播</t>
+          <t>材料完整</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>提交练习产物</t>
+          <t>总部培训教室</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>投影、麦克风、签到二维码</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>场地容量待确认</t>
         </is>
       </c>
     </row>
@@ -10644,32 +10664,40 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>面试官认证培训后勤</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>一线HR</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>结构化面试训练</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>能够独立完成结构化面试训练的基础操作，并说明关键风险边界。</t>
-        </is>
+      <c r="D3" s="2" t="n">
+        <v>30</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>半天</t>
+          <t>线下工作坊</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>线下工作坊</t>
+          <t>缺少证明</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>完成情景演练</t>
+          <t>线上会议室</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>直播链接、录制权限、互动工具</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>线上链接需提前压测</t>
         </is>
       </c>
     </row>
@@ -10681,32 +10709,40 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HRBP</t>
+          <t>绩效宣导会务</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>新员工文化导入</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>能够独立完成新员工文化导入的基础操作，并说明关键风险边界。</t>
-        </is>
+          <t>部门管理者</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>36</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1天</t>
+          <t>混合式学习</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>混合式学习</t>
+          <t>需主管确认</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>通过小测</t>
+          <t>外部会议场地</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>白板、便签、分组桌牌</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>签到数据需脱敏汇总</t>
         </is>
       </c>
     </row>
@@ -10718,32 +10754,40 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>部门管理者</t>
+          <t>线上直播课保障</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>绩效反馈沟通</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>能够独立完成绩效反馈沟通的基础操作，并说明关键风险边界。</t>
-        </is>
+          <t>内训师</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>42</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>2小时</t>
+          <t>自学加答疑</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>自学加答疑</t>
+          <t>尚未上传</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>完成复盘表</t>
+          <t>混合会场</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>考试设备、备用网络</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>设备需准备备用方案</t>
         </is>
       </c>
     </row>
@@ -10755,32 +10799,40 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>内训师</t>
+          <t>线下工作坊物料准备</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>培训项目管理</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>能够独立完成培训项目管理的基础操作，并说明关键风险边界。</t>
-        </is>
+          <t>项目组学员</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>48</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>90分钟</t>
+          <t>线上直播</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>线上直播</t>
+          <t>材料完整</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>提交练习产物</t>
+          <t>总部培训教室</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>投影、麦克风、签到二维码</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>场地容量待确认</t>
         </is>
       </c>
     </row>
@@ -10792,32 +10844,40 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>内训师沙龙签到</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
           <t>新员工</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>政策问答服务</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>能够独立完成政策问答服务的基础操作，并说明关键风险边界。</t>
-        </is>
+      <c r="D7" s="2" t="n">
+        <v>54</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>半天</t>
+          <t>线下工作坊</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>线下工作坊</t>
+          <t>缺少证明</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>完成情景演练</t>
+          <t>线上会议室</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>直播链接、录制权限、互动工具</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>线上链接需提前压测</t>
         </is>
       </c>
     </row>
@@ -10829,32 +10889,40 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>培训考试组织</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
           <t>一线HR</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>会议纪要规范</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>能够独立完成会议纪要规范的基础操作，并说明关键风险边界。</t>
-        </is>
+      <c r="D8" s="2" t="n">
+        <v>60</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1天</t>
+          <t>混合式学习</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>混合式学习</t>
+          <t>需主管确认</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>通过小测</t>
+          <t>外部会议场地</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>白板、便签、分组桌牌</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>签到数据需脱敏汇总</t>
         </is>
       </c>
     </row>
@@ -10866,32 +10934,40 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>HRBP</t>
+          <t>跨城培训会务</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>岗位说明书编写</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>能够独立完成岗位说明书编写的基础操作，并说明关键风险边界。</t>
-        </is>
+          <t>部门管理者</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>66</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>2小时</t>
+          <t>自学加答疑</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>自学加答疑</t>
+          <t>尚未上传</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>完成复盘表</t>
+          <t>混合会场</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>考试设备、备用网络</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>设备需准备备用方案</t>
         </is>
       </c>
     </row>

</xml_diff>